<commit_message>
Correct K105_E121_Dist description and fig_coupling label
K105_E121_Dist uses Pfam Pkinase HMM nodes 62 and 78 (PKA canonical K105
and E121 positions). In CSK, the residue at the K105 position is GLN (not K).
This contact is an alphaC-beta4 loop element, not the beta3-Lys/alphaC-Glu
salt bridge; that is SB_Dist (HMM nodes 30 and 48).

data_dictionary v7r3 and v7r2: updated K105_E121_Dist description to name
the correct HMM nodes and residue identities, and explicitly cross-reference
SB_Dist for the regulatory salt bridge.

fig_coupling.py: display label changed from "b3K-aCE (K105-E121)" to
"alphaC-loop (K105-E121)"; panel B title from "b3K-aCE network" to
"K105-E121 alphaC-loop network".

Assisted-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AlloQuant_master_CSV_data_dictionary_v7r2.xlsx
+++ b/docs/AlloQuant_master_CSV_data_dictionary_v7r2.xlsx
@@ -565,6 +565,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -614,6 +615,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -2414,7 +2416,7 @@
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>Min side-chain distance K105 to E121 (component of the beta3 Lys / alphaC Glu network).</t>
+          <t>Min side-chain distance between residues at Pfam Pkinase HMM node 62 (PKA canonical K105 position; GLN65 in CSK domain numbering) and HMM node 78 (PKA canonical E121 position; GLU82 in CSK domain numbering). Part of the alphaC-beta4 loop contact network. NOT the beta3-Lys/alphaC-Glu regulatory salt bridge -- for that, see SB_Dist.</t>
         </is>
       </c>
     </row>

</xml_diff>